<commit_message>
fix(excel): correct FCF memo row and add interest coverage ratio
</commit_message>
<xml_diff>
--- a/FA583/coursework/RELX_Financial_Analysis_FA583_FINAL.xlsx
+++ b/FA583/coursework/RELX_Financial_Analysis_FA583_FINAL.xlsx
@@ -470,7 +470,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="90">
+  <cellXfs count="91">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -691,6 +691,7 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1105,7 +1106,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="89" t="inlineStr">
+      <c r="A1" s="90" t="inlineStr">
         <is>
           <t>RELX PLC - Income Statement (£m)</t>
         </is>
@@ -1472,7 +1473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -1483,7 +1484,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="89" t="inlineStr">
+      <c r="A1" s="90" t="inlineStr">
         <is>
           <t>RELX PLC - Balance Sheet (£m)</t>
         </is>
@@ -1978,7 +1979,23 @@
       <c r="D36" s="77" t="n"/>
       <c r="E36" s="76" t="n"/>
     </row>
-    <row r="37" ht="15" customHeight="1"/>
+    <row r="37" ht="15" customHeight="1">
+      <c r="A37" s="79" t="inlineStr">
+        <is>
+          <t>MEMO: Net debt</t>
+        </is>
+      </c>
+      <c r="B37" s="80" t="n">
+        <v>6604</v>
+      </c>
+      <c r="C37" s="80" t="n">
+        <v>6446</v>
+      </c>
+      <c r="D37" s="80" t="n">
+        <v>6563</v>
+      </c>
+      <c r="E37" s="81" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:E1"/>
@@ -1993,7 +2010,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D28"/>
+  <dimension ref="A1:D29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -2003,7 +2020,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="89" t="inlineStr">
+      <c r="A1" s="90" t="inlineStr">
         <is>
           <t>RELX PLC - Cash Flow Statement (£m)</t>
         </is>
@@ -2370,7 +2387,22 @@
       <c r="C28" s="77" t="n"/>
       <c r="D28" s="77" t="n"/>
     </row>
-    <row r="29" ht="15" customHeight="1"/>
+    <row r="29" ht="15" customHeight="1">
+      <c r="A29" s="79" t="inlineStr">
+        <is>
+          <t>MEMO: Free cash flow (approx.)</t>
+        </is>
+      </c>
+      <c r="B29" s="81" t="n">
+        <v>1965</v>
+      </c>
+      <c r="C29" s="80" t="n">
+        <v>1980</v>
+      </c>
+      <c r="D29" s="80" t="n">
+        <v>2124</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:D1"/>
@@ -2385,7 +2417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -2406,6 +2438,7 @@
       <c r="C1" s="86" t="n"/>
       <c r="D1" s="86" t="n"/>
       <c r="E1" s="86" t="n"/>
+      <c r="F1" s="88" t="n"/>
     </row>
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="66" t="inlineStr">
@@ -2417,6 +2450,7 @@
       <c r="C2" s="66" t="n"/>
       <c r="D2" s="66" t="n"/>
       <c r="E2" s="66" t="n"/>
+      <c r="F2" s="66" t="n"/>
     </row>
     <row r="3" ht="18" customHeight="1">
       <c r="A3" s="70" t="inlineStr">
@@ -2442,6 +2476,11 @@
       <c r="E3" s="72" t="inlineStr">
         <is>
           <t>Formula</t>
+        </is>
+      </c>
+      <c r="F3" s="72" t="inlineStr">
+        <is>
+          <t>Notes</t>
         </is>
       </c>
     </row>
@@ -2455,6 +2494,7 @@
       <c r="C4" s="63" t="n"/>
       <c r="D4" s="63" t="n"/>
       <c r="E4" s="63" t="n"/>
+      <c r="F4" s="64" t="n"/>
     </row>
     <row r="5" ht="16" customHeight="1">
       <c r="A5" s="70" t="inlineStr">
@@ -2476,6 +2516,11 @@
           <t>EBIT / (Total assets − Current liabilities)</t>
         </is>
       </c>
+      <c r="F5" s="72" t="inlineStr">
+        <is>
+          <t>Capital employed = total assets less current liabilities</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="16" customHeight="1">
       <c r="A6" s="73" t="inlineStr">
@@ -2497,6 +2542,11 @@
           <t>Gross profit / Revenue</t>
         </is>
       </c>
+      <c r="F6" s="75" t="inlineStr">
+        <is>
+          <t>Stable ~65% — subscription cost base is predictable</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="70" t="inlineStr">
@@ -2518,9 +2568,14 @@
           <t>Net profit (shareholders) / Revenue</t>
         </is>
       </c>
+      <c r="F7" s="72" t="inlineStr">
+        <is>
+          <t>Improved despite UK tax rise to 25% (Apr 2023)</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="16" customHeight="1">
-      <c r="A8" s="88" t="inlineStr">
+      <c r="A8" s="89" t="inlineStr">
         <is>
           <t>LIQUIDITY — SHORT-TERM</t>
         </is>
@@ -2529,6 +2584,7 @@
       <c r="C8" s="63" t="n"/>
       <c r="D8" s="63" t="n"/>
       <c r="E8" s="63" t="n"/>
+      <c r="F8" s="64" t="n"/>
     </row>
     <row r="9" ht="16" customHeight="1">
       <c r="A9" s="70" t="inlineStr">
@@ -2550,6 +2606,11 @@
           <t>Current assets / Current liabilities</t>
         </is>
       </c>
+      <c r="F9" s="72" t="inlineStr">
+        <is>
+          <t>Below 1.0x — structural: ~£4bn deferred subscription income in CL</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="16" customHeight="1">
       <c r="A10" s="70" t="inlineStr">
@@ -2571,6 +2632,11 @@
           <t>(Current assets − Inventories) / Current liabilities</t>
         </is>
       </c>
+      <c r="F10" s="72" t="inlineStr">
+        <is>
+          <t>Closely tracks current ratio — minimal inventory effect</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="16" customHeight="1">
       <c r="A11" s="70" t="inlineStr">
@@ -2592,6 +2658,11 @@
           <t>(Inventories / Cost of sales) × 365</t>
         </is>
       </c>
+      <c r="F11" s="72" t="inlineStr">
+        <is>
+          <t>Stable ~37 days — mainly physical exhibition/print inventory</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="16" customHeight="1">
       <c r="A12" s="70" t="inlineStr">
@@ -2613,9 +2684,14 @@
           <t>(Trade receivables / Revenue) × 365</t>
         </is>
       </c>
+      <c r="F12" s="72" t="inlineStr">
+        <is>
+          <t>Long but improving — B2B enterprise clients on annual contracts</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="16" customHeight="1">
-      <c r="A13" s="88" t="inlineStr">
+      <c r="A13" s="89" t="inlineStr">
         <is>
           <t>LIQUIDITY — LONG-TERM / SOLVENCY</t>
         </is>
@@ -2624,6 +2700,7 @@
       <c r="C13" s="63" t="n"/>
       <c r="D13" s="63" t="n"/>
       <c r="E13" s="63" t="n"/>
+      <c r="F13" s="64" t="n"/>
     </row>
     <row r="14" ht="16" customHeight="1">
       <c r="A14" s="70" t="inlineStr">
@@ -2643,6 +2720,37 @@
       <c r="E14" s="72" t="inlineStr">
         <is>
           <t>Long-term borrowings / (Long-term borrowings + Equity)</t>
+        </is>
+      </c>
+      <c r="F14" s="72" t="inlineStr">
+        <is>
+          <t>Elevated but slowly declining; equity base partly intangible</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Interest coverage ratio</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="C15" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="D15" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>EBIT / Finance costs</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Declined to 8.3x in 2023 (higher refinancing cost), recovered to 9.4x in 2024; comfortably covered throughout</t>
         </is>
       </c>
     </row>

</xml_diff>